<commit_message>
Attribute TEMT to the TCI–IIMB lab; re-record the tour with Microsoft's Ava voice
- Every reference to the Supply Chain Management Centre now names the TCI–IIMB Supply
  Chain Sustainability Lab: site header and footer, hero, FAQ, methodology, privacy,
  sign-in page, Copilot answers, PDF reports, structured data and llms.txt. The contact
  links still work but no longer show the SCMC address.
- The tour video is narrated by Microsoft's Ava neural voice (96 kbps) and re-recorded so
  the screens show the new branding.
- Fix: audio.py wrote the mix to out/demo while the render read public/mix.wav, so the
  previous video carried an old narration over newer screens. The mix now goes to
  public/mix.wav, the music pad sits 20 dB under the voice, the chapter whooshes are gone
  and loudness is normalised with one constant gain.
- Video files carry the recording date so no cache serves an earlier cut.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/web/public/downloads/temt-sample-report.xlsx
+++ b/apps/web/public/downloads/temt-sample-report.xlsx
@@ -15641,7 +15641,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{43961080-B250-4593-BF23-F3C1F3785D9B}</x14:id>
+          <x14:id>{7BA921D6-3EBE-4939-93C1-25AA04EDE716}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -15652,7 +15652,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{43961080-B250-4593-BF23-F3C1F3785D9B}">
+          <x14:cfRule type="dataBar" id="{7BA921D6-3EBE-4939-93C1-25AA04EDE716}">
             <x14:dataBar minLength="0" maxLength="100">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>

</xml_diff>